<commit_message>
Initialized paired and single sample workflows
</commit_message>
<xml_diff>
--- a/Example_Paired_Data.xlsx
+++ b/Example_Paired_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pattac/Desktop/DTSEA_git/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55936663-B12B-9744-A2EA-94E2B9D4D67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C71E037-9DA7-8D45-9B0D-50BA3BDBDCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" xr2:uid="{4BB580A1-9C49-44F8-8A9F-9E02B64B4125}"/>
+    <workbookView xWindow="34560" yWindow="3120" windowWidth="32000" windowHeight="17500" xr2:uid="{4BB580A1-9C49-44F8-8A9F-9E02B64B4125}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="2" r:id="rId1"/>
@@ -7528,9 +7528,6 @@
     <t>Mapping_Library</t>
   </si>
   <si>
-    <t>MIPE_5_DSEA_Sets.gmt</t>
-  </si>
-  <si>
     <t>Tests</t>
   </si>
   <si>
@@ -7559,6 +7556,9 @@
   </si>
   <si>
     <t>(Please enter in the same order as they appear in the Data tab. Remove any whitespace from column names)</t>
+  </si>
+  <si>
+    <t>Pharos_DSEA_Sets.gmt</t>
   </si>
 </sst>
 </file>
@@ -7997,7 +7997,7 @@
         <v>2491</v>
       </c>
       <c r="C3" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -8011,22 +8011,22 @@
         <v>92.1</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>2500</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>2501</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>2502</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>2503</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>2504</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>2505</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>2506</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -8108,18 +8108,18 @@
         <v>2496</v>
       </c>
       <c r="B9" t="s">
-        <v>2497</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
+        <v>2497</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2499</v>
+      </c>
+      <c r="C10" t="s">
         <v>2498</v>
-      </c>
-      <c r="B10" t="s">
-        <v>2500</v>
-      </c>
-      <c r="C10" t="s">
-        <v>2499</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -8150,22 +8150,22 @@
         <v>92.1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2500</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2501</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2502</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2503</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2504</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2505</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>2506</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Rename workflows to EDTEA and check paired dependencies
</commit_message>
<xml_diff>
--- a/Example_Paired_Data.xlsx
+++ b/Example_Paired_Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pattac/Desktop/DTSEA_git/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pattac/Desktop/EDTEA_git/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C71E037-9DA7-8D45-9B0D-50BA3BDBDCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -7507,7 +7507,7 @@
     <t>Root_Directory</t>
   </si>
   <si>
-    <t>~/Desktop/DTSEA_git</t>
+    <t>~/Desktop/EDTEA_git</t>
   </si>
   <si>
     <t>Data_Columns</t>

</xml_diff>